<commit_message>
Ajout du réseau PERT, des matrices RACI et parties prenantes, et de l'auto-évaluation
</commit_message>
<xml_diff>
--- a/01-techniques-de-gestion-de-projets/rendu-de-sousa-nunes-alessandro/projet-5-pilotage-complet/plan-et-suivi-du-projet.xlsx
+++ b/01-techniques-de-gestion-de-projets/rendu-de-sousa-nunes-alessandro/projet-5-pilotage-complet/plan-et-suivi-du-projet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0ee8758c4b754eab/Bureau/E3-Gestion-de-projets-PPE/01-techniques-de-gestion-de-projets/rendu-de-sousa-nunes-alessandro/projet-5-pilotage-complet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{86021EC6-7D5C-4367-A41C-31001EC01B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A67A707-5BCD-4DE0-A379-42DAA92C2103}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{86021EC6-7D5C-4367-A41C-31001EC01B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DF0347C-6410-45FA-9194-D2327CE6F71F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{3C127EF1-88B8-41E3-BCCF-74B7726C9B37}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="Planning" sheetId="2" r:id="rId2"/>
     <sheet name="Suivi" sheetId="3" r:id="rId3"/>
     <sheet name="Risques" sheetId="4" r:id="rId4"/>
+    <sheet name="RACI" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="102">
   <si>
     <t>Budget prévisionnel - Mise en place d'un wiki interne</t>
   </si>
@@ -309,13 +310,52 @@
   </si>
   <si>
     <t>SIMULATION : formateur absent, les valeurs réelles (cellules jaunes) sont un cas plausible choisi par le chef de projet. Aléa simulé : administrateur système malade le J3.</t>
+  </si>
+  <si>
+    <t>Matrice RACI - Mise en place du wiki interne</t>
+  </si>
+  <si>
+    <t>Activité</t>
+  </si>
+  <si>
+    <t>Sponsor</t>
+  </si>
+  <si>
+    <t>Utilisateurs</t>
+  </si>
+  <si>
+    <t>Contrôle (un seul A)</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>L3 - Configuration (droits, comptes)</t>
+  </si>
+  <si>
+    <t>Décisions du comité (réserve, aléa)</t>
+  </si>
+  <si>
+    <t>Mise en service et clôture</t>
+  </si>
+  <si>
+    <t>R = Réalise le travail   |   A = Approuve, rend des comptes (un seul par activité)   |   C = Consulté avant   |   I = Informé après</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,6 +413,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFC0392B"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -443,7 +491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -503,11 +551,67 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF008000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF5B25C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC0392B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF3B78B5"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -846,6 +950,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -2127,16 +2235,313 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E9">
-    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
       <formula>$E5&gt;=12</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
       <formula>($E5&gt;=8)*($E5&lt;12)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="3" stopIfTrue="1">
       <formula>$E5&lt;8</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6E985D2-F768-48BB-B550-A821D31698C7}">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="44.6328125" customWidth="1"/>
+    <col min="2" max="8" width="14.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E5" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H5" s="10" t="str">
+        <f>IF(COUNTIF(B5:G5,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="10" t="str">
+        <f>IF(COUNTIF(B6:G6,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="10" t="str">
+        <f>IF(COUNTIF(B7:G7,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="H8" s="10" t="str">
+        <f>IF(COUNTIF(B8:G8,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="H9" s="10" t="str">
+        <f>IF(COUNTIF(B9:G9,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="G10" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="10" t="str">
+        <f>IF(COUNTIF(B10:G10,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" s="30"/>
+      <c r="H11" s="10" t="str">
+        <f>IF(COUNTIF(B11:G11,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="30"/>
+      <c r="H12" s="10" t="str">
+        <f>IF(COUNTIF(B12:G12,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E13" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="F13" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G13" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="H13" s="10" t="str">
+        <f>IF(COUNTIF(B13:G13,"A")=1,"OK","Erreur")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B5:G13">
+    <cfRule type="cellIs" dxfId="4" priority="1" stopIfTrue="1" operator="equal">
+      <formula>"R"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="2" stopIfTrue="1" operator="equal">
+      <formula>"A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="equal">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="4" stopIfTrue="1" operator="equal">
+      <formula>"I"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H13">
+    <cfRule type="cellIs" dxfId="0" priority="5" stopIfTrue="1" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>